<commit_message>
Poprawa formuł workbooka ekologii
</commit_message>
<xml_diff>
--- a/output/Ekologia_kalkulator.xlsx
+++ b/output/Ekologia_kalkulator.xlsx
@@ -1187,7 +1187,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Trend stężeń - Slot 6</a:t>
+              <a:t>Trend stężeń - BENZEN</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -3516,8 +3516,16 @@
           <t>Zanieczyszczenie 6</t>
         </is>
       </c>
-      <c r="B87" s="8" t="inlineStr"/>
-      <c r="C87" s="8" t="inlineStr"/>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>BENZEN</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>benzen</t>
+        </is>
+      </c>
       <c r="D87" s="8" t="inlineStr">
         <is>
           <t>µg/m3</t>
@@ -3556,90 +3564,150 @@
         <f>$B$2+0</f>
         <v/>
       </c>
-      <c r="B89" s="6" t="n"/>
-      <c r="C89" s="6" t="n"/>
-      <c r="D89" s="6" t="n"/>
+      <c r="B89" s="6" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C89" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D89" s="6" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="5">
         <f>$B$2+1</f>
         <v/>
       </c>
-      <c r="B90" s="6" t="n"/>
-      <c r="C90" s="6" t="n"/>
-      <c r="D90" s="6" t="n"/>
+      <c r="B90" s="6" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="C90" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D90" s="6" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="5">
         <f>$B$2+2</f>
         <v/>
       </c>
-      <c r="B91" s="6" t="n"/>
-      <c r="C91" s="6" t="n"/>
-      <c r="D91" s="6" t="n"/>
+      <c r="B91" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C91" s="6" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D91" s="6" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="5">
         <f>$B$2+3</f>
         <v/>
       </c>
-      <c r="B92" s="6" t="n"/>
-      <c r="C92" s="6" t="n"/>
-      <c r="D92" s="6" t="n"/>
+      <c r="B92" s="6" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C92" s="6" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D92" s="6" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="5">
         <f>$B$2+4</f>
         <v/>
       </c>
-      <c r="B93" s="6" t="n"/>
-      <c r="C93" s="6" t="n"/>
-      <c r="D93" s="6" t="n"/>
+      <c r="B93" s="6" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="C93" s="6" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D93" s="6" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="5">
         <f>$B$2+5</f>
         <v/>
       </c>
-      <c r="B94" s="6" t="n"/>
-      <c r="C94" s="6" t="n"/>
-      <c r="D94" s="6" t="n"/>
+      <c r="B94" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C94" s="6" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D94" s="6" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="5">
         <f>$B$2+6</f>
         <v/>
       </c>
-      <c r="B95" s="6" t="n"/>
-      <c r="C95" s="6" t="n"/>
-      <c r="D95" s="6" t="n"/>
+      <c r="B95" s="6" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="C95" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D95" s="6" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="5">
         <f>$B$2+7</f>
         <v/>
       </c>
-      <c r="B96" s="6" t="n"/>
-      <c r="C96" s="6" t="n"/>
-      <c r="D96" s="6" t="n"/>
+      <c r="B96" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C96" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D96" s="6" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="5">
         <f>$B$2+8</f>
         <v/>
       </c>
-      <c r="B97" s="6" t="n"/>
-      <c r="C97" s="6" t="n"/>
-      <c r="D97" s="6" t="n"/>
+      <c r="B97" s="6" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C97" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D97" s="6" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="5">
         <f>$B$2+9</f>
         <v/>
       </c>
-      <c r="B98" s="6" t="n"/>
-      <c r="C98" s="6" t="n"/>
-      <c r="D98" s="6" t="n"/>
+      <c r="B98" s="6" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="C98" s="6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D98" s="6" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
@@ -4549,15 +4617,15 @@
         <v/>
       </c>
       <c r="J10" s="12">
-        <f>IF(COUNTA(B14:B23)=0,"",MIN(B14:B23))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B14:B23)=0,"",MIN('Powietrze_Dane'!B14:B23))</f>
         <v/>
       </c>
       <c r="K10" s="12">
-        <f>IF(COUNTA(B14:B23)=0,"",AVERAGE(B14:B23))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B14:B23)=0,"",AVERAGE('Powietrze_Dane'!B14:B23))</f>
         <v/>
       </c>
       <c r="L10" s="12">
-        <f>IF(COUNTA(B14:B23)=0,"",MAX(B14:B23))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B14:B23)=0,"",MAX('Powietrze_Dane'!B14:B23))</f>
         <v/>
       </c>
       <c r="M10" s="12">
@@ -4636,15 +4704,15 @@
         <v/>
       </c>
       <c r="J11" s="12">
-        <f>IF(COUNTA(C14:C23)=0,"",MIN(C14:C23))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C14:C23)=0,"",MIN('Powietrze_Dane'!C14:C23))</f>
         <v/>
       </c>
       <c r="K11" s="12">
-        <f>IF(COUNTA(C14:C23)=0,"",AVERAGE(C14:C23))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C14:C23)=0,"",AVERAGE('Powietrze_Dane'!C14:C23))</f>
         <v/>
       </c>
       <c r="L11" s="12">
-        <f>IF(COUNTA(C14:C23)=0,"",MAX(C14:C23))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C14:C23)=0,"",MAX('Powietrze_Dane'!C14:C23))</f>
         <v/>
       </c>
       <c r="M11" s="12">
@@ -4723,15 +4791,15 @@
         <v/>
       </c>
       <c r="J12" s="12">
-        <f>IF(COUNTA(D14:D23)=0,"",MIN(D14:D23))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D14:D23)=0,"",MIN('Powietrze_Dane'!D14:D23))</f>
         <v/>
       </c>
       <c r="K12" s="12">
-        <f>IF(COUNTA(D14:D23)=0,"",AVERAGE(D14:D23))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D14:D23)=0,"",AVERAGE('Powietrze_Dane'!D14:D23))</f>
         <v/>
       </c>
       <c r="L12" s="12">
-        <f>IF(COUNTA(D14:D23)=0,"",MAX(D14:D23))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D14:D23)=0,"",MAX('Powietrze_Dane'!D14:D23))</f>
         <v/>
       </c>
       <c r="M12" s="12">
@@ -4810,15 +4878,15 @@
         <v/>
       </c>
       <c r="J13" s="12">
-        <f>IF(COUNTA(B29:B38)=0,"",MIN(B29:B38))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B29:B38)=0,"",MIN('Powietrze_Dane'!B29:B38))</f>
         <v/>
       </c>
       <c r="K13" s="12">
-        <f>IF(COUNTA(B29:B38)=0,"",AVERAGE(B29:B38))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B29:B38)=0,"",AVERAGE('Powietrze_Dane'!B29:B38))</f>
         <v/>
       </c>
       <c r="L13" s="12">
-        <f>IF(COUNTA(B29:B38)=0,"",MAX(B29:B38))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B29:B38)=0,"",MAX('Powietrze_Dane'!B29:B38))</f>
         <v/>
       </c>
       <c r="M13" s="12">
@@ -4897,15 +4965,15 @@
         <v/>
       </c>
       <c r="J14" s="12">
-        <f>IF(COUNTA(C29:C38)=0,"",MIN(C29:C38))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C29:C38)=0,"",MIN('Powietrze_Dane'!C29:C38))</f>
         <v/>
       </c>
       <c r="K14" s="12">
-        <f>IF(COUNTA(C29:C38)=0,"",AVERAGE(C29:C38))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C29:C38)=0,"",AVERAGE('Powietrze_Dane'!C29:C38))</f>
         <v/>
       </c>
       <c r="L14" s="12">
-        <f>IF(COUNTA(C29:C38)=0,"",MAX(C29:C38))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C29:C38)=0,"",MAX('Powietrze_Dane'!C29:C38))</f>
         <v/>
       </c>
       <c r="M14" s="12">
@@ -4984,15 +5052,15 @@
         <v/>
       </c>
       <c r="J15" s="12">
-        <f>IF(COUNTA(D29:D38)=0,"",MIN(D29:D38))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D29:D38)=0,"",MIN('Powietrze_Dane'!D29:D38))</f>
         <v/>
       </c>
       <c r="K15" s="12">
-        <f>IF(COUNTA(D29:D38)=0,"",AVERAGE(D29:D38))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D29:D38)=0,"",AVERAGE('Powietrze_Dane'!D29:D38))</f>
         <v/>
       </c>
       <c r="L15" s="12">
-        <f>IF(COUNTA(D29:D38)=0,"",MAX(D29:D38))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D29:D38)=0,"",MAX('Powietrze_Dane'!D29:D38))</f>
         <v/>
       </c>
       <c r="M15" s="12">
@@ -5071,15 +5139,15 @@
         <v/>
       </c>
       <c r="J16" s="12">
-        <f>IF(COUNTA(B44:B53)=0,"",MIN(B44:B53))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B44:B53)=0,"",MIN('Powietrze_Dane'!B44:B53))</f>
         <v/>
       </c>
       <c r="K16" s="12">
-        <f>IF(COUNTA(B44:B53)=0,"",AVERAGE(B44:B53))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B44:B53)=0,"",AVERAGE('Powietrze_Dane'!B44:B53))</f>
         <v/>
       </c>
       <c r="L16" s="12">
-        <f>IF(COUNTA(B44:B53)=0,"",MAX(B44:B53))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B44:B53)=0,"",MAX('Powietrze_Dane'!B44:B53))</f>
         <v/>
       </c>
       <c r="M16" s="12">
@@ -5158,15 +5226,15 @@
         <v/>
       </c>
       <c r="J17" s="12">
-        <f>IF(COUNTA(C44:C53)=0,"",MIN(C44:C53))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C44:C53)=0,"",MIN('Powietrze_Dane'!C44:C53))</f>
         <v/>
       </c>
       <c r="K17" s="12">
-        <f>IF(COUNTA(C44:C53)=0,"",AVERAGE(C44:C53))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C44:C53)=0,"",AVERAGE('Powietrze_Dane'!C44:C53))</f>
         <v/>
       </c>
       <c r="L17" s="12">
-        <f>IF(COUNTA(C44:C53)=0,"",MAX(C44:C53))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C44:C53)=0,"",MAX('Powietrze_Dane'!C44:C53))</f>
         <v/>
       </c>
       <c r="M17" s="12">
@@ -5245,15 +5313,15 @@
         <v/>
       </c>
       <c r="J18" s="12">
-        <f>IF(COUNTA(D44:D53)=0,"",MIN(D44:D53))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D44:D53)=0,"",MIN('Powietrze_Dane'!D44:D53))</f>
         <v/>
       </c>
       <c r="K18" s="12">
-        <f>IF(COUNTA(D44:D53)=0,"",AVERAGE(D44:D53))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D44:D53)=0,"",AVERAGE('Powietrze_Dane'!D44:D53))</f>
         <v/>
       </c>
       <c r="L18" s="12">
-        <f>IF(COUNTA(D44:D53)=0,"",MAX(D44:D53))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D44:D53)=0,"",MAX('Powietrze_Dane'!D44:D53))</f>
         <v/>
       </c>
       <c r="M18" s="12">
@@ -5332,15 +5400,15 @@
         <v/>
       </c>
       <c r="J19" s="12">
-        <f>IF(COUNTA(B59:B68)=0,"",MIN(B59:B68))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B59:B68)=0,"",MIN('Powietrze_Dane'!B59:B68))</f>
         <v/>
       </c>
       <c r="K19" s="12">
-        <f>IF(COUNTA(B59:B68)=0,"",AVERAGE(B59:B68))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B59:B68)=0,"",AVERAGE('Powietrze_Dane'!B59:B68))</f>
         <v/>
       </c>
       <c r="L19" s="12">
-        <f>IF(COUNTA(B59:B68)=0,"",MAX(B59:B68))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B59:B68)=0,"",MAX('Powietrze_Dane'!B59:B68))</f>
         <v/>
       </c>
       <c r="M19" s="12">
@@ -5419,15 +5487,15 @@
         <v/>
       </c>
       <c r="J20" s="12">
-        <f>IF(COUNTA(C59:C68)=0,"",MIN(C59:C68))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C59:C68)=0,"",MIN('Powietrze_Dane'!C59:C68))</f>
         <v/>
       </c>
       <c r="K20" s="12">
-        <f>IF(COUNTA(C59:C68)=0,"",AVERAGE(C59:C68))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C59:C68)=0,"",AVERAGE('Powietrze_Dane'!C59:C68))</f>
         <v/>
       </c>
       <c r="L20" s="12">
-        <f>IF(COUNTA(C59:C68)=0,"",MAX(C59:C68))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C59:C68)=0,"",MAX('Powietrze_Dane'!C59:C68))</f>
         <v/>
       </c>
       <c r="M20" s="12">
@@ -5506,15 +5574,15 @@
         <v/>
       </c>
       <c r="J21" s="12">
-        <f>IF(COUNTA(D59:D68)=0,"",MIN(D59:D68))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D59:D68)=0,"",MIN('Powietrze_Dane'!D59:D68))</f>
         <v/>
       </c>
       <c r="K21" s="12">
-        <f>IF(COUNTA(D59:D68)=0,"",AVERAGE(D59:D68))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D59:D68)=0,"",AVERAGE('Powietrze_Dane'!D59:D68))</f>
         <v/>
       </c>
       <c r="L21" s="12">
-        <f>IF(COUNTA(D59:D68)=0,"",MAX(D59:D68))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D59:D68)=0,"",MAX('Powietrze_Dane'!D59:D68))</f>
         <v/>
       </c>
       <c r="M21" s="12">
@@ -5593,15 +5661,15 @@
         <v/>
       </c>
       <c r="J22" s="12">
-        <f>IF(COUNTA(B74:B83)=0,"",MIN(B74:B83))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B74:B83)=0,"",MIN('Powietrze_Dane'!B74:B83))</f>
         <v/>
       </c>
       <c r="K22" s="12">
-        <f>IF(COUNTA(B74:B83)=0,"",AVERAGE(B74:B83))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B74:B83)=0,"",AVERAGE('Powietrze_Dane'!B74:B83))</f>
         <v/>
       </c>
       <c r="L22" s="12">
-        <f>IF(COUNTA(B74:B83)=0,"",MAX(B74:B83))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B74:B83)=0,"",MAX('Powietrze_Dane'!B74:B83))</f>
         <v/>
       </c>
       <c r="M22" s="12">
@@ -5680,15 +5748,15 @@
         <v/>
       </c>
       <c r="J23" s="12">
-        <f>IF(COUNTA(C74:C83)=0,"",MIN(C74:C83))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C74:C83)=0,"",MIN('Powietrze_Dane'!C74:C83))</f>
         <v/>
       </c>
       <c r="K23" s="12">
-        <f>IF(COUNTA(C74:C83)=0,"",AVERAGE(C74:C83))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C74:C83)=0,"",AVERAGE('Powietrze_Dane'!C74:C83))</f>
         <v/>
       </c>
       <c r="L23" s="12">
-        <f>IF(COUNTA(C74:C83)=0,"",MAX(C74:C83))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C74:C83)=0,"",MAX('Powietrze_Dane'!C74:C83))</f>
         <v/>
       </c>
       <c r="M23" s="12">
@@ -5767,15 +5835,15 @@
         <v/>
       </c>
       <c r="J24" s="12">
-        <f>IF(COUNTA(D74:D83)=0,"",MIN(D74:D83))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D74:D83)=0,"",MIN('Powietrze_Dane'!D74:D83))</f>
         <v/>
       </c>
       <c r="K24" s="12">
-        <f>IF(COUNTA(D74:D83)=0,"",AVERAGE(D74:D83))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D74:D83)=0,"",AVERAGE('Powietrze_Dane'!D74:D83))</f>
         <v/>
       </c>
       <c r="L24" s="12">
-        <f>IF(COUNTA(D74:D83)=0,"",MAX(D74:D83))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D74:D83)=0,"",MAX('Powietrze_Dane'!D74:D83))</f>
         <v/>
       </c>
       <c r="M24" s="12">
@@ -5854,15 +5922,15 @@
         <v/>
       </c>
       <c r="J25" s="12">
-        <f>IF(COUNTA(B89:B98)=0,"",MIN(B89:B98))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B89:B98)=0,"",MIN('Powietrze_Dane'!B89:B98))</f>
         <v/>
       </c>
       <c r="K25" s="12">
-        <f>IF(COUNTA(B89:B98)=0,"",AVERAGE(B89:B98))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B89:B98)=0,"",AVERAGE('Powietrze_Dane'!B89:B98))</f>
         <v/>
       </c>
       <c r="L25" s="12">
-        <f>IF(COUNTA(B89:B98)=0,"",MAX(B89:B98))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!B89:B98)=0,"",MAX('Powietrze_Dane'!B89:B98))</f>
         <v/>
       </c>
       <c r="M25" s="12">
@@ -5941,15 +6009,15 @@
         <v/>
       </c>
       <c r="J26" s="12">
-        <f>IF(COUNTA(C89:C98)=0,"",MIN(C89:C98))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C89:C98)=0,"",MIN('Powietrze_Dane'!C89:C98))</f>
         <v/>
       </c>
       <c r="K26" s="12">
-        <f>IF(COUNTA(C89:C98)=0,"",AVERAGE(C89:C98))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C89:C98)=0,"",AVERAGE('Powietrze_Dane'!C89:C98))</f>
         <v/>
       </c>
       <c r="L26" s="12">
-        <f>IF(COUNTA(C89:C98)=0,"",MAX(C89:C98))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!C89:C98)=0,"",MAX('Powietrze_Dane'!C89:C98))</f>
         <v/>
       </c>
       <c r="M26" s="12">
@@ -6028,15 +6096,15 @@
         <v/>
       </c>
       <c r="J27" s="12">
-        <f>IF(COUNTA(D89:D98)=0,"",MIN(D89:D98))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D89:D98)=0,"",MIN('Powietrze_Dane'!D89:D98))</f>
         <v/>
       </c>
       <c r="K27" s="12">
-        <f>IF(COUNTA(D89:D98)=0,"",AVERAGE(D89:D98))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D89:D98)=0,"",AVERAGE('Powietrze_Dane'!D89:D98))</f>
         <v/>
       </c>
       <c r="L27" s="12">
-        <f>IF(COUNTA(D89:D98)=0,"",MAX(D89:D98))</f>
+        <f>IF(COUNTA('Powietrze_Dane'!D89:D98)=0,"",MAX('Powietrze_Dane'!D89:D98))</f>
         <v/>
       </c>
       <c r="M27" s="12">
@@ -6899,7 +6967,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>Gleba_Wyniki!B5</f>
+        <f>Gleba_Wyniki!B4</f>
         <v/>
       </c>
     </row>
@@ -6910,7 +6978,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>Gleba_Wyniki!B6</f>
+        <f>Gleba_Wyniki!B5</f>
         <v/>
       </c>
     </row>
@@ -6921,7 +6989,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>Gleba_Wyniki!B7</f>
+        <f>Gleba_Wyniki!B6</f>
         <v/>
       </c>
     </row>
@@ -6932,7 +7000,7 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>Gleba_Wyniki!B8</f>
+        <f>Gleba_Wyniki!B7</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Poprawa liczników pominiec w workbooku Excel
</commit_message>
<xml_diff>
--- a/output/Ekologia_kalkulator.xlsx
+++ b/output/Ekologia_kalkulator.xlsx
@@ -4383,11 +4383,11 @@
         <v/>
       </c>
       <c r="H3" s="12">
-        <f>COUNTIFS($B$10:$B$27,A3,$Q$10:$Q$27,"&lt;&gt;")</f>
+        <f>SUMPRODUCT(($B$10:$B$27=A3)*(LEN($Q$10:$Q$27)&gt;0))</f>
         <v/>
       </c>
       <c r="I3" s="12">
-        <f>COUNTIFS($B$10:$B$27,A3,$R$10:$R$27,"&lt;&gt;")</f>
+        <f>SUMPRODUCT(($B$10:$B$27=A3)*(LEN($R$10:$R$27)&gt;0))</f>
         <v/>
       </c>
     </row>
@@ -4422,11 +4422,11 @@
         <v/>
       </c>
       <c r="H4" s="12">
-        <f>COUNTIFS($B$10:$B$27,A4,$Q$10:$Q$27,"&lt;&gt;")</f>
+        <f>SUMPRODUCT(($B$10:$B$27=A4)*(LEN($Q$10:$Q$27)&gt;0))</f>
         <v/>
       </c>
       <c r="I4" s="12">
-        <f>COUNTIFS($B$10:$B$27,A4,$R$10:$R$27,"&lt;&gt;")</f>
+        <f>SUMPRODUCT(($B$10:$B$27=A4)*(LEN($R$10:$R$27)&gt;0))</f>
         <v/>
       </c>
     </row>
@@ -4461,11 +4461,11 @@
         <v/>
       </c>
       <c r="H5" s="12">
-        <f>COUNTIFS($B$10:$B$27,A5,$Q$10:$Q$27,"&lt;&gt;")</f>
+        <f>SUMPRODUCT(($B$10:$B$27=A5)*(LEN($Q$10:$Q$27)&gt;0))</f>
         <v/>
       </c>
       <c r="I5" s="12">
-        <f>COUNTIFS($B$10:$B$27,A5,$R$10:$R$27,"&lt;&gt;")</f>
+        <f>SUMPRODUCT(($B$10:$B$27=A5)*(LEN($R$10:$R$27)&gt;0))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Poprawa nagłówków arkusza mapowania powietrza
</commit_message>
<xml_diff>
--- a/output/Ekologia_kalkulator.xlsx
+++ b/output/Ekologia_kalkulator.xlsx
@@ -3759,12 +3759,12 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Zanieczyszczenie</t>
+          <t>Substancja</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Współczynnik toksyczności</t>
+          <t>Limit D24 [µg/m3]</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">

</xml_diff>